<commit_message>
Presentation-only polish: Hindi labels for codes, 2-bedroom callout
No data refreshed, no external call: re-rendered offline from the saved
final dataset. Hindi files show classification codes as natural Hindi
labels with the code in parentheses (e.g. कुल मासिक खर्च बजट के भीतर
(STRICT_ALL_IN)). Both executive PDFs gain an informational
'Best 2-bedroom options' callout (top 3 collected 2BR, existing rank
order; Top 10 unchanged). English workbook and both contact templates
are byte-identical; EN/HI parity checks pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jr5gB4bHTzGs4KWP2Fpqrg
</commit_message>
<xml_diff>
--- a/outputs/Miraflores_Rental_Shortlist_HI.xlsx
+++ b/outputs/Miraflores_Rental_Shortlist_HI.xlsx
@@ -1792,7 +1792,7 @@
   <autoFilter ref="A4:N14"/>
   <conditionalFormatting sqref="A5:N14">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -2047,9 +2047,9 @@
       <c r="G5" s="6" t="n">
         <v>855.24</v>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I5" s="4" t="n">
@@ -2109,9 +2109,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V5" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W5" s="11" t="inlineStr">
@@ -2134,14 +2134,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA5" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB5" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2173,9 +2173,9 @@
       <c r="G6" s="6" t="n">
         <v>886.26</v>
       </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I6" s="4" t="n">
@@ -2233,9 +2233,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V6" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -2258,14 +2258,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA6" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB6" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2297,9 +2297,9 @@
       <c r="G7" s="6" t="n">
         <v>992.62</v>
       </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I7" s="4" t="n">
@@ -2357,9 +2357,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V7" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W7" s="11" t="inlineStr">
@@ -2382,14 +2382,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA7" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB7" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2421,9 +2421,9 @@
       <c r="G8" s="6" t="n">
         <v>827.17</v>
       </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I8" s="4" t="n">
@@ -2483,9 +2483,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V8" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -2508,14 +2508,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA8" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB8" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2547,9 +2547,9 @@
       <c r="G9" s="6" t="n">
         <v>753.33</v>
       </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I9" s="4" t="n">
@@ -2609,9 +2609,9 @@
           <t>मुख्य सड़क (आर्टेरियल) पर स्थित (शोर का प्रमाण देखें) — बेडरूम में ट्रैफ़िक का शोर ज़रूर जाँचें</t>
         </is>
       </c>
-      <c r="V9" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -2634,14 +2634,14 @@
           <t>नक्शा देखें</t>
         </is>
       </c>
-      <c r="AA9" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB9" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2673,9 +2673,9 @@
       <c r="G10" s="6" t="n">
         <v>983.75</v>
       </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I10" s="4" t="n">
@@ -2735,9 +2735,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V10" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W10" s="11" t="inlineStr">
@@ -2760,14 +2760,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA10" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB10" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2799,9 +2799,9 @@
       <c r="G11" s="6" t="n">
         <v>798.23</v>
       </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I11" s="4" t="n">
@@ -2859,9 +2859,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V11" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W11" s="11" t="inlineStr">
@@ -2884,14 +2884,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA11" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB11" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -2923,9 +2923,9 @@
       <c r="G12" s="6" t="n">
         <v>832.49</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I12" s="4" t="n">
@@ -2983,9 +2983,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V12" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W12" s="11" t="inlineStr">
@@ -3008,14 +3008,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA12" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB12" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -3047,9 +3047,9 @@
       <c r="G13" s="6" t="n">
         <v>983.75</v>
       </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I13" s="4" t="n">
@@ -3111,9 +3111,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V13" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -3136,14 +3136,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA13" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA13" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB13" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -3175,9 +3175,9 @@
       <c r="G14" s="6" t="n">
         <v>815.36</v>
       </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I14" s="4" t="n">
@@ -3239,9 +3239,9 @@
           <t>असुसज्जित</t>
         </is>
       </c>
-      <c r="V14" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -3264,14 +3264,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA14" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AB14" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
     </row>
@@ -3303,9 +3303,9 @@
       <c r="G15" s="6" t="n">
         <v>971.9400000000001</v>
       </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I15" s="4" t="n">
@@ -3367,9 +3367,9 @@
           <t>असुसज्जित</t>
         </is>
       </c>
-      <c r="V15" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W15" s="11" t="inlineStr">
@@ -3392,14 +3392,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA15" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB15" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA15" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I16" s="4" t="n">
@@ -3493,9 +3493,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,099 (USD 996 किराया + S/ 350 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V16" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -3518,14 +3518,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA16" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB16" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA16" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I17" s="4" t="n">
@@ -3617,9 +3617,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,100 (USD 996 किराया + S/ 350 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V17" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W17" s="5" t="inlineStr">
@@ -3642,14 +3642,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA17" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB17" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA17" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB17" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I18" s="4" t="n">
@@ -3747,9 +3747,9 @@
           <t>रखरखाव शुल्क प्रकाशित नहीं — देखने जाने से पहले पुष्टि करें</t>
         </is>
       </c>
-      <c r="V18" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -3772,14 +3772,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA18" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB18" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA18" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB18" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -3811,9 +3811,9 @@
       <c r="G19" s="6" t="n">
         <v>903.99</v>
       </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I19" s="4" t="n">
@@ -3875,9 +3875,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V19" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W19" s="5" t="inlineStr">
@@ -3900,14 +3900,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA19" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB19" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA19" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB19" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I20" s="4" t="n">
@@ -4001,9 +4001,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,072 (USD 994 किराया + S/ 265 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V20" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -4026,14 +4026,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA20" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB20" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA20" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB20" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4065,9 +4065,9 @@
       <c r="G21" s="6" t="n">
         <v>732.65</v>
       </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="I21" s="4" t="n">
@@ -4127,9 +4127,9 @@
           <t>नक्शे पर स्थान नहीं — शोर का अनुमान केवल विज्ञापन के विवरण पर आधारित</t>
         </is>
       </c>
-      <c r="V21" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W21" s="11" t="inlineStr">
@@ -4152,14 +4152,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA21" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB21" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA21" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB21" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I22" s="4" t="n">
@@ -4251,9 +4251,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,001 (USD 919 किराया + S/ 280 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V22" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -4276,14 +4276,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA22" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB22" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA22" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB22" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I23" s="4" t="n">
@@ -4379,9 +4379,9 @@
           <t>मुख्य सड़क (आर्टेरियल) पर स्थित (शोर का प्रमाण देखें) — बेडरूम में ट्रैफ़िक का शोर ज़रूर जाँचें</t>
         </is>
       </c>
-      <c r="V23" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W23" s="11" t="inlineStr">
@@ -4404,14 +4404,14 @@
           <t>नक्शा देखें</t>
         </is>
       </c>
-      <c r="AA23" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB23" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA23" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB23" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I24" s="4" t="n">
@@ -4503,9 +4503,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,108 (USD 975 किराया + S/ 450 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V24" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W24" s="11" t="inlineStr">
@@ -4528,14 +4528,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA24" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB24" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA24" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB24" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I25" s="4" t="n">
@@ -4629,9 +4629,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,005 (USD 896 किराया + S/ 370 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V25" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W25" s="11" t="inlineStr">
@@ -4654,14 +4654,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA25" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB25" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA25" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB25" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I26" s="4" t="n">
@@ -4755,9 +4755,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,049 (USD 940 किराया + S/ 370 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V26" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W26" s="11" t="inlineStr">
@@ -4780,14 +4780,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA26" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB26" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA26" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB26" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="I27" s="4" t="n">
@@ -4881,9 +4881,9 @@
           <t>किराया + रखरखाव शुल्क ≈ USD 1,105 (USD 999 किराया + S/ 360 रखरखाव शुल्क) — USD 1,000 से अधिक</t>
         </is>
       </c>
-      <c r="V27" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="V27" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="W27" s="11" t="inlineStr">
@@ -4906,14 +4906,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="AA27" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
-        </is>
-      </c>
-      <c r="AB27" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="AA27" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
+        </is>
+      </c>
+      <c r="AB27" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
   <autoFilter ref="A4:AB27"/>
   <conditionalFormatting sqref="A5:AB27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="0">
       <formula>AND($A5="शीर्ष 10",$B5&lt;=5)</formula>
@@ -4956,10 +4956,10 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H27">
     <cfRule type="expression" priority="9" dxfId="3" stopIfTrue="1">
-      <formula>H5="STRICT_ALL_IN"</formula>
+      <formula>H5="कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="8" stopIfTrue="1">
-      <formula>H5="BASE_RENT_COMPLIANT"</formula>
+      <formula>H5="मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C27">
@@ -5393,9 +5393,9 @@
           <t>1BR · 62 m² — Miraflores · ID 151162497</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr"/>
@@ -5407,9 +5407,9 @@
           <t>PEN 2,600</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I5" s="15" t="n">
@@ -5420,17 +5420,17 @@
           <t>S/ 295 (≈ USD 87)</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L5" s="6" t="n">
         <v>855.24</v>
       </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr">
@@ -5454,15 +5454,15 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T5" s="14" t="n">
         <v>12.39</v>
       </c>
-      <c r="U5" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V5" s="11" t="inlineStr">
@@ -5563,9 +5563,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP5" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ5" s="5" t="inlineStr">
@@ -5580,12 +5580,12 @@
       </c>
       <c r="AS5" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT5" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU5" s="11" t="inlineStr">
@@ -5632,14 +5632,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE5" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF5" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG5" s="5" t="inlineStr">
@@ -5660,9 +5660,9 @@
           <t>1BR · 42 m² — Miraflores · ID 151122912</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr"/>
@@ -5674,9 +5674,9 @@
           <t>PEN 2,800</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I6" s="15" t="n">
@@ -5687,17 +5687,17 @@
           <t>S/ 200 (≈ USD 59)</t>
         </is>
       </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L6" s="6" t="n">
         <v>886.26</v>
       </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N6" s="11" t="inlineStr">
@@ -5719,9 +5719,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S6" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T6" s="14" t="n">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V6" s="11" t="inlineStr">
@@ -5828,9 +5828,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP6" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP6" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ6" s="5" t="inlineStr">
@@ -5845,12 +5845,12 @@
       </c>
       <c r="AS6" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; STUDIO_WORDING</t>
-        </is>
-      </c>
-      <c r="AT6" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); स्टूडियो जैसा विवरण (STUDIO_WORDING)</t>
+        </is>
+      </c>
+      <c r="AT6" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU6" s="5" t="inlineStr">
@@ -5897,14 +5897,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE6" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE6" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF6" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG6" s="5" t="inlineStr">
@@ -5925,9 +5925,9 @@
           <t>1BR · 71 m² — Miraflores · ID 150746422</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr"/>
@@ -5939,9 +5939,9 @@
           <t>PEN 3,060</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I7" s="15" t="n">
@@ -5952,17 +5952,17 @@
           <t>S/ 300 (≈ USD 89)</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L7" s="6" t="n">
         <v>992.62</v>
       </c>
-      <c r="M7" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr">
@@ -5986,15 +5986,15 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T7" s="14" t="n">
         <v>12.73</v>
       </c>
-      <c r="U7" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V7" s="11" t="inlineStr">
@@ -6093,9 +6093,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP7" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP7" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ7" s="5" t="inlineStr">
@@ -6110,12 +6110,12 @@
       </c>
       <c r="AS7" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT7" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT7" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU7" s="11" t="inlineStr">
@@ -6162,14 +6162,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE7" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE7" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF7" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG7" s="5" t="inlineStr">
@@ -6190,9 +6190,9 @@
           <t>1BR · 40 m² — San Antonio</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr"/>
@@ -6204,9 +6204,9 @@
           <t>PEN 2,600</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I8" s="15" t="n">
@@ -6217,17 +6217,17 @@
           <t>S/ 200 (≈ USD 59)</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L8" s="6" t="n">
         <v>827.17</v>
       </c>
-      <c r="M8" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N8" s="11" t="inlineStr">
@@ -6249,17 +6249,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S8" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T8" s="14" t="n">
         <v>19.2</v>
       </c>
-      <c r="U8" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V8" s="11" t="inlineStr">
@@ -6360,9 +6360,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP8" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP8" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ8" s="5" t="inlineStr">
@@ -6377,12 +6377,12 @@
       </c>
       <c r="AS8" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT8" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT8" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU8" s="11" t="inlineStr">
@@ -6429,14 +6429,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE8" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE8" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF8" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG8" s="5" t="inlineStr">
@@ -6457,9 +6457,9 @@
           <t>1BR · 41 m² — Miraflores · ID 151178161</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr"/>
@@ -6471,9 +6471,9 @@
           <t>PEN 2,300</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I9" s="15" t="n">
@@ -6484,17 +6484,17 @@
           <t>S/ 250 (≈ USD 74)</t>
         </is>
       </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L9" s="6" t="n">
         <v>753.33</v>
       </c>
-      <c r="M9" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N9" s="11" t="inlineStr">
@@ -6516,17 +6516,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S9" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T9" s="14" t="n">
         <v>16.57</v>
       </c>
-      <c r="U9" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V9" s="5" t="inlineStr">
@@ -6621,9 +6621,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP9" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP9" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ9" s="5" t="inlineStr">
@@ -6638,12 +6638,12 @@
       </c>
       <c r="AS9" s="5" t="inlineStr">
         <is>
-          <t>APPROXIMATE_LOCATION; DIRECT_MAJOR_AVENUE; INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_PUBLICATION_DATE; ON_MAJOR_ARTERIAL; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT9" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>अनुमानित स्थान (APPROXIMATE_LOCATION); मुख्य एवेन्यू के बिल्कुल पास (DIRECT_MAJOR_AVENUE); पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); मुख्य सड़क पर (ON_MAJOR_ARTERIAL); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT9" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU9" s="11" t="inlineStr">
@@ -6692,12 +6692,12 @@
       </c>
       <c r="BE9" s="5" t="inlineStr">
         <is>
-          <t>GEOCODED_TEXT / STREET_LEVEL</t>
+          <t>विज्ञापन के पते से (GEOCODED_TEXT) / सड़क-स्तर (STREET_LEVEL)</t>
         </is>
       </c>
       <c r="BF9" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG9" s="5" t="inlineStr">
@@ -6718,9 +6718,9 @@
           <t>1BR · 71 m² — Miraflores · ID 150877601</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr"/>
@@ -6732,9 +6732,9 @@
           <t>PEN 3,000</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I10" s="15" t="n">
@@ -6745,17 +6745,17 @@
           <t>S/ 330 (≈ USD 97)</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L10" s="6" t="n">
         <v>983.75</v>
       </c>
-      <c r="M10" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N10" s="11" t="inlineStr">
@@ -6779,15 +6779,15 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T10" s="14" t="n">
         <v>12.48</v>
       </c>
-      <c r="U10" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V10" s="11" t="inlineStr">
@@ -6888,9 +6888,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP10" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP10" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ10" s="5" t="inlineStr">
@@ -6905,12 +6905,12 @@
       </c>
       <c r="AS10" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT10" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT10" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU10" s="5" t="inlineStr">
@@ -6957,14 +6957,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE10" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE10" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF10" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG10" s="5" t="inlineStr">
@@ -6985,9 +6985,9 @@
           <t>1BR · 45 m² — Miraflores · ID 146109648</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr"/>
@@ -6999,9 +6999,9 @@
           <t>PEN 2,452</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I11" s="15" t="n">
@@ -7012,17 +7012,17 @@
           <t>S/ 250 (≈ USD 74)</t>
         </is>
       </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L11" s="6" t="n">
         <v>798.23</v>
       </c>
-      <c r="M11" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr">
@@ -7044,17 +7044,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S11" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T11" s="14" t="n">
         <v>16.1</v>
       </c>
-      <c r="U11" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V11" s="11" t="inlineStr">
@@ -7153,9 +7153,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP11" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP11" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ11" s="5" t="inlineStr">
@@ -7170,12 +7170,12 @@
       </c>
       <c r="AS11" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; STUDIO_WORDING</t>
-        </is>
-      </c>
-      <c r="AT11" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); स्टूडियो जैसा विवरण (STUDIO_WORDING)</t>
+        </is>
+      </c>
+      <c r="AT11" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU11" s="11" t="inlineStr">
@@ -7222,14 +7222,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE11" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE11" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF11" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG11" s="5" t="inlineStr">
@@ -7250,9 +7250,9 @@
           <t>1BR · 43 m² — Miraflores · ID 151124896</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr"/>
@@ -7264,9 +7264,9 @@
           <t>PEN 2,528</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I12" s="15" t="n">
@@ -7277,17 +7277,17 @@
           <t>S/ 290 (≈ USD 86)</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L12" s="6" t="n">
         <v>832.49</v>
       </c>
-      <c r="M12" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N12" s="11" t="inlineStr">
@@ -7309,17 +7309,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S12" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T12" s="14" t="n">
         <v>17.37</v>
       </c>
-      <c r="U12" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V12" s="11" t="inlineStr">
@@ -7418,9 +7418,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP12" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP12" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ12" s="5" t="inlineStr">
@@ -7435,12 +7435,12 @@
       </c>
       <c r="AS12" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT12" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT12" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU12" s="5" t="inlineStr">
@@ -7487,14 +7487,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE12" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE12" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF12" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG12" s="5" t="inlineStr">
@@ -7515,9 +7515,9 @@
           <t>1BR · 71 m² — Miraflores · ID 150869056</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr"/>
@@ -7529,9 +7529,9 @@
           <t>PEN 3,000</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I13" s="15" t="n">
@@ -7542,17 +7542,17 @@
           <t>S/ 330 (≈ USD 97)</t>
         </is>
       </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L13" s="6" t="n">
         <v>983.75</v>
       </c>
-      <c r="M13" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N13" s="11" t="inlineStr">
@@ -7576,15 +7576,15 @@
       </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T13" s="14" t="n">
         <v>12.48</v>
       </c>
-      <c r="U13" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V13" s="11" t="inlineStr">
@@ -7687,9 +7687,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP13" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP13" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ13" s="5" t="inlineStr">
@@ -7704,12 +7704,12 @@
       </c>
       <c r="AS13" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT13" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT13" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU13" s="11" t="inlineStr">
@@ -7756,14 +7756,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE13" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE13" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF13" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG13" s="5" t="inlineStr">
@@ -7784,9 +7784,9 @@
           <t>2BR · 96 m² — Miraflores · ID 151159973</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr"/>
@@ -7798,9 +7798,9 @@
           <t>PEN 2,500</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I14" s="15" t="n">
@@ -7811,17 +7811,17 @@
           <t>S/ 260 (≈ USD 77)</t>
         </is>
       </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L14" s="6" t="n">
         <v>815.36</v>
       </c>
-      <c r="M14" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N14" s="11" t="inlineStr">
@@ -7845,15 +7845,15 @@
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T14" s="14" t="n">
         <v>7.69</v>
       </c>
-      <c r="U14" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V14" s="11" t="inlineStr">
@@ -7956,9 +7956,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP14" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP14" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ14" s="5" t="inlineStr">
@@ -7973,12 +7973,12 @@
       </c>
       <c r="AS14" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_FURNITURE; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT14" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); असुसज्जित (NO_FURNITURE); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT14" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU14" s="11" t="inlineStr">
@@ -8025,14 +8025,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE14" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
+      <c r="BE14" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
         </is>
       </c>
       <c r="BF14" s="5" t="inlineStr">
         <is>
-          <t>UNVERIFIED_NOT_RETURNED</t>
+          <t>पुनः-जाँच में पुष्टि नहीं हो सकी (UNVERIFIED_NOT_RETURNED)</t>
         </is>
       </c>
       <c r="BG14" s="5" t="inlineStr">
@@ -8053,9 +8053,9 @@
           <t>2BR · 95 m² — Miraflores · ID 151011858</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr"/>
@@ -8067,9 +8067,9 @@
           <t>PEN 2,890</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I15" s="15" t="n">
@@ -8080,17 +8080,17 @@
           <t>S/ 400 (≈ USD 118)</t>
         </is>
       </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L15" s="6" t="n">
         <v>971.9400000000001</v>
       </c>
-      <c r="M15" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N15" s="11" t="inlineStr">
@@ -8114,15 +8114,15 @@
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T15" s="14" t="n">
         <v>8.99</v>
       </c>
-      <c r="U15" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V15" s="11" t="inlineStr">
@@ -8225,9 +8225,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP15" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP15" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ15" s="5" t="inlineStr">
@@ -8242,12 +8242,12 @@
       </c>
       <c r="AS15" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_FURNITURE; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT15" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); असुसज्जित (NO_FURNITURE); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT15" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU15" s="11" t="inlineStr">
@@ -8294,14 +8294,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE15" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF15" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE15" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF15" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG15" s="11" t="inlineStr">
@@ -8322,9 +8322,9 @@
           <t>2BR · 80 m² — Miraflores · ID 150982482</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr"/>
@@ -8336,9 +8336,9 @@
           <t>PEN 3,370</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I16" s="15" t="n">
@@ -8349,9 +8349,9 @@
           <t>S/ 350 (≈ USD 103)</t>
         </is>
       </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L16" s="6" t="n">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
@@ -8381,17 +8381,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S16" s="11" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा (GOOD)</t>
         </is>
       </c>
       <c r="T16" s="14" t="n">
         <v>12.44</v>
       </c>
-      <c r="U16" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V16" s="11" t="inlineStr">
@@ -8492,9 +8492,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP16" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP16" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ16" s="5" t="inlineStr">
@@ -8509,12 +8509,12 @@
       </c>
       <c r="AS16" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT16" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT16" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU16" s="5" t="inlineStr">
@@ -8561,14 +8561,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE16" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF16" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE16" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF16" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG16" s="11" t="inlineStr">
@@ -8589,9 +8589,9 @@
           <t>2BR · 87 m² — Miraflores · ID 151058338</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr"/>
@@ -8603,9 +8603,9 @@
           <t>PEN 3,373</t>
         </is>
       </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I17" s="15" t="n">
@@ -8616,9 +8616,9 @@
           <t>S/ 350 (≈ USD 103)</t>
         </is>
       </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L17" s="6" t="n">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
@@ -8650,15 +8650,15 @@
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T17" s="14" t="n">
         <v>11.45</v>
       </c>
-      <c r="U17" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V17" s="11" t="inlineStr">
@@ -8757,9 +8757,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP17" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP17" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ17" s="5" t="inlineStr">
@@ -8774,12 +8774,12 @@
       </c>
       <c r="AS17" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT17" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT17" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU17" s="11" t="inlineStr">
@@ -8826,14 +8826,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE17" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF17" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE17" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF17" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG17" s="11" t="inlineStr">
@@ -8854,9 +8854,9 @@
           <t>1BR · 68 m² — Miraflores · ID 150518776</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr"/>
@@ -8868,9 +8868,9 @@
           <t>PEN 3,000</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I18" s="15" t="n">
@@ -8881,9 +8881,9 @@
           <t>जानकारी उपलब्ध नहीं</t>
         </is>
       </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -8893,7 +8893,7 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
@@ -8917,15 +8917,15 @@
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T18" s="14" t="n">
         <v>13.03</v>
       </c>
-      <c r="U18" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -9028,9 +9028,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP18" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP18" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ18" s="5" t="inlineStr">
@@ -9045,12 +9045,12 @@
       </c>
       <c r="AS18" s="5" t="inlineStr">
         <is>
-          <t>CURRENCY_CONVERSION_MISMATCH; INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; UNKNOWN_MAINTENANCE</t>
-        </is>
-      </c>
-      <c r="AT18" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>मुद्रा-रूपांतरण में अंतर (CURRENCY_CONVERSION_MISMATCH); पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); रखरखाव शुल्क अज्ञात (UNKNOWN_MAINTENANCE)</t>
+        </is>
+      </c>
+      <c r="AT18" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU18" s="11" t="inlineStr">
@@ -9097,14 +9097,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE18" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF18" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE18" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF18" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG18" s="11" t="inlineStr">
@@ -9125,9 +9125,9 @@
           <t>1BR · 40 m² — Alexander Von Humboldt</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr"/>
@@ -9139,9 +9139,9 @@
           <t>PEN 2,800</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I19" s="15" t="n">
@@ -9152,17 +9152,17 @@
           <t>S/ 260 (≈ USD 77)</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L19" s="6" t="n">
         <v>903.99</v>
       </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N19" s="11" t="inlineStr">
@@ -9184,9 +9184,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S19" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T19" s="14" t="n">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V19" s="5" t="inlineStr">
@@ -9297,9 +9297,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP19" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP19" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ19" s="11" t="inlineStr">
@@ -9314,12 +9314,12 @@
       </c>
       <c r="AS19" s="5" t="inlineStr">
         <is>
-          <t>CURRENCY_CONVERSION_MISMATCH; INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN</t>
-        </is>
-      </c>
-      <c r="AT19" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>मुद्रा-रूपांतरण में अंतर (CURRENCY_CONVERSION_MISMATCH); पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN)</t>
+        </is>
+      </c>
+      <c r="AT19" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU19" s="11" t="inlineStr">
@@ -9366,14 +9366,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE19" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF19" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE19" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF19" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG19" s="11" t="inlineStr">
@@ -9394,9 +9394,9 @@
           <t>2BR · 65 m² — Miraflores · ID 151047474</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr"/>
@@ -9408,9 +9408,9 @@
           <t>PEN 3,365</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I20" s="15" t="n">
@@ -9421,9 +9421,9 @@
           <t>S/ 265 (≈ USD 78)</t>
         </is>
       </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L20" s="6" t="n">
@@ -9431,7 +9431,7 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
@@ -9453,9 +9453,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S20" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T20" s="14" t="n">
@@ -9463,7 +9463,7 @@
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V20" s="11" t="inlineStr">
@@ -9564,9 +9564,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP20" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP20" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ20" s="5" t="inlineStr">
@@ -9581,12 +9581,12 @@
       </c>
       <c r="AS20" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT20" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT20" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU20" s="5" t="inlineStr">
@@ -9633,14 +9633,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE20" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF20" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE20" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF20" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG20" s="11" t="inlineStr">
@@ -9661,9 +9661,9 @@
           <t>1BR · 39 m² — Miraflores · ID 150752635</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr"/>
@@ -9675,9 +9675,9 @@
           <t>PEN 2,200</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I21" s="15" t="n">
@@ -9688,17 +9688,17 @@
           <t>S/ 280 (≈ USD 83)</t>
         </is>
       </c>
-      <c r="K21" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L21" s="6" t="n">
         <v>732.65</v>
       </c>
-      <c r="M21" s="11" t="inlineStr">
-        <is>
-          <t>STRICT_ALL_IN</t>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)</t>
         </is>
       </c>
       <c r="N21" s="11" t="inlineStr">
@@ -9720,17 +9720,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S21" s="11" t="inlineStr">
-        <is>
-          <t>SMALL</t>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>छोटा (SMALL)</t>
         </is>
       </c>
       <c r="T21" s="14" t="n">
         <v>16.66</v>
       </c>
-      <c r="U21" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V21" s="5" t="inlineStr">
@@ -9831,9 +9831,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP21" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP21" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ21" s="5" t="inlineStr">
@@ -9848,12 +9848,12 @@
       </c>
       <c r="AS21" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; STUDIO_WORDING</t>
-        </is>
-      </c>
-      <c r="AT21" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); स्टूडियो जैसा विवरण (STUDIO_WORDING)</t>
+        </is>
+      </c>
+      <c r="AT21" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU21" s="5" t="inlineStr">
@@ -9900,14 +9900,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE21" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF21" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE21" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF21" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG21" s="11" t="inlineStr">
@@ -9928,9 +9928,9 @@
           <t>2BR · 81 m² — Miraflores · ID 151167358</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr"/>
@@ -9942,9 +9942,9 @@
           <t>PEN 3,110</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I22" s="15" t="n">
@@ -9955,9 +9955,9 @@
           <t>S/ 280 (≈ USD 83)</t>
         </is>
       </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L22" s="6" t="n">
@@ -9965,7 +9965,7 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
@@ -9987,17 +9987,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S22" s="11" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा (GOOD)</t>
         </is>
       </c>
       <c r="T22" s="14" t="n">
         <v>11.34</v>
       </c>
-      <c r="U22" s="11" t="inlineStr">
-        <is>
-          <t>GOOD_VALUE</t>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा मूल्य (GOOD_VALUE)</t>
         </is>
       </c>
       <c r="V22" s="11" t="inlineStr">
@@ -10096,9 +10096,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP22" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP22" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ22" s="5" t="inlineStr">
@@ -10113,12 +10113,12 @@
       </c>
       <c r="AS22" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_FURNITURE; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT22" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); असुसज्जित (NO_FURNITURE); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT22" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU22" s="5" t="inlineStr">
@@ -10165,14 +10165,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE22" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF22" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE22" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF22" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG22" s="11" t="inlineStr">
@@ -10193,9 +10193,9 @@
           <t>2BR · 79 m² — Miraflores · ID 149641202</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr"/>
@@ -10207,9 +10207,9 @@
           <t>PEN 3,360</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I23" s="15" t="n">
@@ -10220,9 +10220,9 @@
           <t>जानकारी उपलब्ध नहीं</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -10232,7 +10232,7 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
@@ -10254,17 +10254,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S23" s="11" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा (GOOD)</t>
         </is>
       </c>
       <c r="T23" s="14" t="n">
         <v>12.56</v>
       </c>
-      <c r="U23" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V23" s="5" t="inlineStr">
@@ -10359,9 +10359,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP23" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP23" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ23" s="5" t="inlineStr">
@@ -10376,12 +10376,12 @@
       </c>
       <c r="AS23" s="5" t="inlineStr">
         <is>
-          <t>APPROXIMATE_LOCATION; DIRECT_MAJOR_AVENUE; HIGH_NOISE_RISK; INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_PUBLICATION_DATE; ON_MAJOR_ARTERIAL; PRICE_CONVERTED_FROM_PEN; UNKNOWN_MAINTENANCE</t>
-        </is>
-      </c>
-      <c r="AT23" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>अनुमानित स्थान (APPROXIMATE_LOCATION); मुख्य एवेन्यू के बिल्कुल पास (DIRECT_MAJOR_AVENUE); शोर का अधिक जोखिम (HIGH_NOISE_RISK); पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); मुख्य सड़क पर (ON_MAJOR_ARTERIAL); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); रखरखाव शुल्क अज्ञात (UNKNOWN_MAINTENANCE)</t>
+        </is>
+      </c>
+      <c r="AT23" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU23" s="11" t="inlineStr">
@@ -10430,12 +10430,12 @@
       </c>
       <c r="BE23" s="5" t="inlineStr">
         <is>
-          <t>GEOCODED_TEXT / STREET_LEVEL</t>
-        </is>
-      </c>
-      <c r="BF23" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+          <t>विज्ञापन के पते से (GEOCODED_TEXT) / सड़क-स्तर (STREET_LEVEL)</t>
+        </is>
+      </c>
+      <c r="BF23" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG23" s="11" t="inlineStr">
@@ -10456,9 +10456,9 @@
           <t>2BR · 95 m² — Miraflores · ID 150634895</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr"/>
@@ -10470,9 +10470,9 @@
           <t>PEN 3,300</t>
         </is>
       </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I24" s="15" t="n">
@@ -10483,9 +10483,9 @@
           <t>S/ 450 (≈ USD 133)</t>
         </is>
       </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L24" s="6" t="n">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
@@ -10517,15 +10517,15 @@
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T24" s="14" t="n">
         <v>10.26</v>
       </c>
-      <c r="U24" s="11" t="inlineStr">
-        <is>
-          <t>EXCELLENT_VALUE</t>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>उत्कृष्ट मूल्य (EXCELLENT_VALUE)</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
@@ -10624,9 +10624,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP24" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP24" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ24" s="5" t="inlineStr">
@@ -10641,12 +10641,12 @@
       </c>
       <c r="AS24" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT24" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT24" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU24" s="5" t="inlineStr">
@@ -10693,14 +10693,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE24" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF24" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE24" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF24" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG24" s="11" t="inlineStr">
@@ -10721,9 +10721,9 @@
           <t>2BR · 60 m² — Miraflores · ID 150773832</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr"/>
@@ -10735,9 +10735,9 @@
           <t>PEN 3,033</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I25" s="15" t="n">
@@ -10748,9 +10748,9 @@
           <t>S/ 370 (≈ USD 109)</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L25" s="6" t="n">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
@@ -10780,9 +10780,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S25" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T25" s="14" t="n">
@@ -10790,7 +10790,7 @@
       </c>
       <c r="U25" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V25" s="5" t="inlineStr">
@@ -10891,9 +10891,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP25" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP25" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ25" s="5" t="inlineStr">
@@ -10908,12 +10908,12 @@
       </c>
       <c r="AS25" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT25" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT25" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU25" s="11" t="inlineStr">
@@ -10960,14 +10960,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE25" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF25" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE25" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF25" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG25" s="11" t="inlineStr">
@@ -10988,9 +10988,9 @@
           <t>2BR · 63 m² — Miraflores · ID 149904784</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr"/>
@@ -11002,9 +11002,9 @@
           <t>PEN 3,182</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I26" s="15" t="n">
@@ -11015,9 +11015,9 @@
           <t>S/ 370 (≈ USD 109)</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L26" s="6" t="n">
@@ -11025,7 +11025,7 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
@@ -11047,17 +11047,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S26" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T26" s="14" t="n">
         <v>14.92</v>
       </c>
-      <c r="U26" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V26" s="11" t="inlineStr">
@@ -11158,9 +11158,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP26" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP26" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ26" s="5" t="inlineStr">
@@ -11175,12 +11175,12 @@
       </c>
       <c r="AS26" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_FURNITURE; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT26" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); असुसज्जित (NO_FURNITURE); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT26" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU26" s="11" t="inlineStr">
@@ -11227,14 +11227,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE26" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF26" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE26" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF26" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG26" s="11" t="inlineStr">
@@ -11255,9 +11255,9 @@
           <t>2BR · 65 m² — Malecon Reserva</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>बजट के भीतर (PRIMARY)</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr"/>
@@ -11269,9 +11269,9 @@
           <t>PEN 3,380</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I27" s="15" t="n">
@@ -11282,9 +11282,9 @@
           <t>S/ 360 (≈ USD 106)</t>
         </is>
       </c>
-      <c r="K27" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L27" s="6" t="n">
@@ -11292,7 +11292,7 @@
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>BASE_RENT_COMPLIANT</t>
+          <t>मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)</t>
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
@@ -11314,9 +11314,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S27" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T27" s="14" t="n">
@@ -11324,7 +11324,7 @@
       </c>
       <c r="U27" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V27" s="11" t="inlineStr">
@@ -11425,9 +11425,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP27" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP27" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ27" s="5" t="inlineStr">
@@ -11442,12 +11442,12 @@
       </c>
       <c r="AS27" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_FURNITURE; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT27" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); असुसज्जित (NO_FURNITURE); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT27" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU27" s="11" t="inlineStr">
@@ -11494,14 +11494,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE27" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF27" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE27" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF27" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG27" s="11" t="inlineStr">
@@ -11514,7 +11514,7 @@
   <autoFilter ref="A4:BG27"/>
   <conditionalFormatting sqref="A5:BG27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="2">
       <formula>MOD(ROW(),2)=0</formula>
@@ -11546,10 +11546,10 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="M5:M27">
     <cfRule type="expression" priority="8" dxfId="3" stopIfTrue="1">
-      <formula>M5="STRICT_ALL_IN"</formula>
+      <formula>M5="कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="8" stopIfTrue="1">
-      <formula>M5="BASE_RENT_COMPLIANT"</formula>
+      <formula>M5="मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B27">
@@ -11983,9 +11983,9 @@
           <t>2BR · 72 m² — Miraflores · ID 151077958</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>STRETCH</t>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>अतिरिक्त बजट / मोलभाव योग्य (STRETCH)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12001,9 +12001,9 @@
           <t>PEN 3,400</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I5" s="15" t="n">
@@ -12014,17 +12014,17 @@
           <t>S/ 420 (≈ USD 124)</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L5" s="6" t="n">
         <v>1128.51</v>
       </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>STRETCH</t>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>अतिरिक्त बजट / मोलभाव योग्य (STRETCH)</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
@@ -12046,17 +12046,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S5" s="11" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>अच्छा (GOOD)</t>
         </is>
       </c>
       <c r="T5" s="14" t="n">
         <v>13.95</v>
       </c>
-      <c r="U5" s="11" t="inlineStr">
-        <is>
-          <t>FAIR_VALUE</t>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>उचित मूल्य (FAIR_VALUE)</t>
         </is>
       </c>
       <c r="V5" s="11" t="inlineStr">
@@ -12155,9 +12155,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP5" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ5" s="5" t="inlineStr">
@@ -12172,12 +12172,12 @@
       </c>
       <c r="AS5" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; MAJOR_ARTERIAL_MENTIONED; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; PRICE_OVER_BUDGET; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT5" s="11" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); पास में मुख्य सड़क का उल्लेख (MAJOR_ARTERIAL_MENTIONED); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); किराया बजट से अधिक (PRICE_OVER_BUDGET); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT5" s="5" t="inlineStr">
+        <is>
+          <t>मध्यम (MEDIUM)</t>
         </is>
       </c>
       <c r="AU5" s="5" t="inlineStr">
@@ -12224,14 +12224,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE5" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF5" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF5" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG5" s="11" t="inlineStr">
@@ -12252,9 +12252,9 @@
           <t>2BR · 60 m² — Miraflores · ID 151047414</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>STRETCH</t>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>अतिरिक्त बजट / मोलभाव योग्य (STRETCH)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12270,9 +12270,9 @@
           <t>PEN 3,540</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I6" s="15" t="n">
@@ -12283,17 +12283,17 @@
           <t>S/ 350 (≈ USD 103)</t>
         </is>
       </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L6" s="6" t="n">
         <v>1149.19</v>
       </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>STRETCH</t>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>अतिरिक्त बजट / मोलभाव योग्य (STRETCH)</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -12315,9 +12315,9 @@
           <t>total</t>
         </is>
       </c>
-      <c r="S6" s="11" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त (ACCEPTABLE)</t>
         </is>
       </c>
       <c r="T6" s="14" t="n">
@@ -12325,7 +12325,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE_RELATIVE_TO_SAMPLE</t>
+          <t>नमूने की तुलना में महँगा (EXPENSIVE_RELATIVE_TO_SAMPLE)</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
@@ -12426,9 +12426,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP6" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP6" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ6" s="5" t="inlineStr">
@@ -12443,12 +12443,12 @@
       </c>
       <c r="AS6" s="5" t="inlineStr">
         <is>
-          <t>INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; POSSIBLE_DUPLICATE; PRICE_CONVERTED_FROM_PEN; PRICE_OVER_BUDGET; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT6" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); संभावित डुप्लिकेट (POSSIBLE_DUPLICATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); किराया बजट से अधिक (PRICE_OVER_BUDGET); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT6" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU6" s="11" t="inlineStr">
@@ -12495,14 +12495,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE6" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF6" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE6" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF6" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG6" s="11" t="inlineStr">
@@ -12515,7 +12515,7 @@
   <autoFilter ref="A4:BG6"/>
   <conditionalFormatting sqref="A5:BG6">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="2">
       <formula>MOD(ROW(),2)=0</formula>
@@ -12547,10 +12547,10 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="M5:M6">
     <cfRule type="expression" priority="8" dxfId="3" stopIfTrue="1">
-      <formula>M5="STRICT_ALL_IN"</formula>
+      <formula>M5="कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="8" stopIfTrue="1">
-      <formula>M5="BASE_RENT_COMPLIANT"</formula>
+      <formula>M5="मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B6">
@@ -12961,9 +12961,9 @@
           <t>1BR · 93 m² — Miraflores · ID 150439988</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>BORDERLINE</t>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>सीमा-रेखा विकल्प (BORDERLINE)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12979,9 +12979,9 @@
           <t>PEN 3,740</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>CALCULATED</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>गणना से (CALCULATED)</t>
         </is>
       </c>
       <c r="I5" s="15" t="n">
@@ -12992,17 +12992,17 @@
           <t>S/ 350 (≈ USD 103)</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>प्रकाशित (PUBLISHED)</t>
         </is>
       </c>
       <c r="L5" s="6" t="n">
         <v>1208.27</v>
       </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>BORDERLINE</t>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>सीमा-रेखा विकल्प (BORDERLINE)</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
@@ -13026,15 +13026,15 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>VERY_SPACIOUS</t>
+          <t>बहुत विशाल (VERY_SPACIOUS)</t>
         </is>
       </c>
       <c r="T5" s="14" t="n">
         <v>11.88</v>
       </c>
-      <c r="U5" s="11" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT_DATA</t>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>पर्याप्त जानकारी नहीं (INSUFFICIENT_DATA)</t>
         </is>
       </c>
       <c r="V5" s="11" t="inlineStr">
@@ -13133,9 +13133,9 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="AP5" s="11" t="inlineStr">
-        <is>
-          <t>LIKELY_ACTIVE</t>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>संभवतः उपलब्ध (LIKELY_ACTIVE)</t>
         </is>
       </c>
       <c r="AQ5" s="5" t="inlineStr">
@@ -13150,12 +13150,12 @@
       </c>
       <c r="AS5" s="5" t="inlineStr">
         <is>
-          <t>BORDERLINE_OVER_STRETCH; INCOMPLETE_ADDRESS; INCOMPLETE_CONTACT; NO_COORDINATES; NO_PUBLICATION_DATE; PRICE_CONVERTED_FROM_PEN; PRICE_OVER_BUDGET; TOTAL_COST_OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="AT5" s="11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
+          <t>स्ट्रेच सीमा से थोड़ा ऊपर (BORDERLINE_OVER_STRETCH); पूरा पता नहीं (INCOMPLETE_ADDRESS); सीधा संपर्क नहीं (INCOMPLETE_CONTACT); नक्शे पर स्थान नहीं (NO_COORDINATES); प्रकाशन तिथि नहीं (NO_PUBLICATION_DATE); किराया PEN से बदला गया (PRICE_CONVERTED_FROM_PEN); किराया बजट से अधिक (PRICE_OVER_BUDGET); कुल खर्च बजट से अधिक (TOTAL_COST_OVER_BUDGET)</t>
+        </is>
+      </c>
+      <c r="AT5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (UNKNOWN)</t>
         </is>
       </c>
       <c r="AU5" s="11" t="inlineStr">
@@ -13202,14 +13202,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="BE5" s="11" t="inlineStr">
-        <is>
-          <t>none / -</t>
-        </is>
-      </c>
-      <c r="BF5" s="11" t="inlineStr">
-        <is>
-          <t>PROGRAMMATIC_WARN</t>
+      <c r="BE5" s="5" t="inlineStr">
+        <is>
+          <t>जानकारी उपलब्ध नहीं (none) / -</t>
+        </is>
+      </c>
+      <c r="BF5" s="5" t="inlineStr">
+        <is>
+          <t>स्वचालित जाँच — ध्यान दें (PROGRAMMATIC_WARN)</t>
         </is>
       </c>
       <c r="BG5" s="11" t="inlineStr">
@@ -13222,7 +13222,7 @@
   <autoFilter ref="A4:BG5"/>
   <conditionalFormatting sqref="A5:BG5">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="2">
       <formula>MOD(ROW(),2)=0</formula>
@@ -13254,10 +13254,10 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="M5">
     <cfRule type="expression" priority="8" dxfId="3" stopIfTrue="1">
-      <formula>M5="STRICT_ALL_IN"</formula>
+      <formula>M5="कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="8" stopIfTrue="1">
-      <formula>M5="BASE_RENT_COMPLIANT"</formula>
+      <formula>M5="मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5">
@@ -13391,9 +13391,9 @@
           <t>Urbania</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>APPROVED</t>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>स्वीकृत (APPROVED)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -13461,9 +13461,9 @@
           <t>Adondevivir</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>APPROVED</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>स्वीकृत (APPROVED)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -13531,9 +13531,9 @@
           <t>Mercado Libre Inmuebles Perú</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>अस्वीकृत (REJECTED)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -13601,9 +13601,9 @@
           <t>Manual import (agency sites, other portals)</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>उपयोग नहीं हुआ (SKIPPED)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
   <autoFilter ref="A4:N16"/>
   <conditionalFormatting sqref="A5:N16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="2">
       <formula>MOD(ROW(),2)=0</formula>
@@ -14300,7 +14300,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>STRICT_ALL_IN = किराया + ज्ञात रखरखाव शुल्क ≤ USD 1,000 · BASE_RENT_COMPLIANT = किराया ≤ USD 1,000, पर कुल खर्च USD 1,000 से अधिक या अज्ञात · STRETCH = किराया USD 1,001–1,100 (अलग शीट) · BORDERLINE = मुद्रा-रूपांतरण के बाद USD 1,100 से अधिकतम 1% ऊपर (लगभग उपयुक्त शीट; कभी बजट के भीतर नहीं)। STRICT_ALL_IN को रैंकिंग में 5 अंकों की प्राथमिकता मिलती है।</t>
+          <t>कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN) = किराया + ज्ञात रखरखाव शुल्क ≤ USD 1,000 · मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT) = किराया ≤ USD 1,000, पर कुल खर्च USD 1,000 से अधिक या अज्ञात · अतिरिक्त बजट / मोलभाव योग्य (STRETCH) = किराया USD 1,001–1,100 (अलग शीट) · सीमा-रेखा विकल्प (BORDERLINE) = मुद्रा-रूपांतरण के बाद USD 1,100 से अधिकतम 1% ऊपर (लगभग उपयुक्त शीट; कभी बजट के भीतर नहीं)। कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN) को रैंकिंग में 5 अंकों की प्राथमिकता मिलती है।</t>
         </is>
       </c>
     </row>
@@ -14348,7 +14348,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>1 USD = S/ 3.385 · BCRP series PD04640PD (SBS sell rate), period 23.Set.26 — https://estadisticas.bcrp.gob.pe/estadisticas/series/api/PD04640PD/json/2026-09-11/2026-09-25/ing · 2026-09-24T20:49:33-05:00। हर रूपांतरण के लिए एक ही दर। बजट, रैंकिंग, USD/m² और कुल खर्च के लिए एक तुलनीय USD मान: USD में दिए किराये के लिए वही USD, अन्यथा PEN ÷ यह दर (CALCULATED)। पोर्टल का अपना USD आँकड़ा अलग रखा गया है; 5% से अधिक अंतर पर CURRENCY_CONVERSION_MISMATCH चिह्न।</t>
+          <t>1 USD = S/ 3.385 · BCRP series PD04640PD (SBS sell rate), period 23.Set.26 — https://estadisticas.bcrp.gob.pe/estadisticas/series/api/PD04640PD/json/2026-09-11/2026-09-25/ing · 2026-09-24T20:36:52-05:00। हर रूपांतरण के लिए एक ही दर। बजट, रैंकिंग, USD/m² और कुल खर्च के लिए एक तुलनीय USD मान: USD में दिए किराये के लिए वही USD, अन्यथा PEN ÷ यह दर (CALCULATED)। पोर्टल का अपना USD आँकड़ा अलग रखा गया है; 5% से अधिक अंतर पर मुद्रा-रूपांतरण में अंतर (CURRENCY_CONVERSION_MISMATCH) चिह्न।</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14408,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>केवल विज्ञापन के विवरण से: HIGH (विदेशियों/पासपोर्ट/कंपनी-अनुबंध का स्पष्ट स्वागत), MEDIUM (अस्थायी अवधि, गारंटर नहीं, अंग्रेज़ी विज्ञापन, सुसज्जित + सेवाएँ शामिल), POTENTIAL_FRICTION (पेरू के गारंटर, carné de extranjería या DNI की माँग), UNKNOWN (कोई उल्लेख नहीं — सामान्य स्थिति, कोई नकारात्मक अंक नहीं)। उल्लेख न होने पर पासपोर्ट की स्वीकार्यता, carné de extranjería, आय का प्रमाण, गारंटर (aval), जमा राशि और न्यूनतम अवधि की पुष्टि करें।</t>
+          <t>केवल विज्ञापन के विवरण से: उच्च (HIGH) = विदेशियों/पासपोर्ट/कंपनी-अनुबंध का स्पष्ट स्वागत; मध्यम (MEDIUM) = अस्थायी अवधि, गारंटर नहीं, अंग्रेज़ी विज्ञापन, सुसज्जित + सेवाएँ शामिल; संभावित अतिरिक्त शर्तें (POTENTIAL_FRICTION) = पेरू के गारंटर, carné de extranjería या DNI की माँग; जानकारी उपलब्ध नहीं (UNKNOWN) = कोई उल्लेख नहीं — सामान्य स्थिति, कोई नकारात्मक अंक नहीं। उल्लेख न होने पर पासपोर्ट की स्वीकार्यता, carné de extranjería, आय का प्रमाण, गारंटर (aval), जमा राशि और न्यूनतम अवधि की पुष्टि करें।</t>
         </is>
       </c>
     </row>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>ACTIVE_CONFIRMED = अंतिम शीर्ष-10 पुनः-जाँच में विज्ञापन सफलतापूर्वक दोबारा खुला · LIKELY_ACTIVE = लाइव खोज में मिला, स्वचालित पुनः-जाँच संभव नहीं (पोर्टल की बॉट-सुरक्षा) · UNKNOWN = पुष्टि नहीं। कभी गारंटी नहीं दी गई।</t>
+          <t>उपलब्धता की पुष्टि हुई (ACTIVE_CONFIRMED) = अंतिम शीर्ष-10 पुनः-जाँच में विज्ञापन सफलतापूर्वक दोबारा खुला · संभवतः उपलब्ध (LIKELY_ACTIVE) = लाइव खोज में मिला, स्वचालित पुनः-जाँच संभव नहीं (पोर्टल की बॉट-सुरक्षा) · जानकारी उपलब्ध नहीं (UNKNOWN) = पुष्टि नहीं। कभी गारंटी नहीं दी गई।</t>
         </is>
       </c>
     </row>
@@ -14444,7 +14444,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>वर्गीकरण कोड अंग्रेज़ी और हिंदी फ़ाइलों में एक जैसे रखे गए हैं: STRICT_ALL_IN, BASE_RENT_COMPLIANT, STRETCH, BORDERLINE (बजट) · ACTIVE_CONFIRMED, LIKELY_ACTIVE, UNKNOWN (उपलब्धता) · HIGH, MEDIUM, POTENTIAL_FRICTION, UNKNOWN (विदेशी किरायेदार) · PUBLISHED / CALCULATED (विज्ञापन में प्रकाशित या रूपांतरित मान) · चेतावनी कोड, जैसे UNKNOWN_MAINTENANCE (रखरखाव शुल्क प्रकाशित नहीं), NO_COORDINATES (नक्शे पर स्थान नहीं), ON_MAJOR_ARTERIAL (पता मुख्य सड़क पर)।</t>
+          <t>हर श्रेणी का हिंदी नाम दिया गया है और अंग्रेज़ी फ़ाइल से मिलान के लिए मूल कोड कोष्ठक में रखा गया है — बजट: कुल मासिक खर्च बजट के भीतर (STRICT_ALL_IN), मूल किराया बजट के भीतर (BASE_RENT_COMPLIANT), अतिरिक्त बजट / मोलभाव योग्य (STRETCH), सीमा-रेखा विकल्प (BORDERLINE); उपलब्धता: उपलब्धता की पुष्टि हुई (ACTIVE_CONFIRMED), संभवतः उपलब्ध (LIKELY_ACTIVE), जानकारी उपलब्ध नहीं (UNKNOWN); विदेशी किरायेदार: उच्च (HIGH), मध्यम (MEDIUM), संभावित अतिरिक्त शर्तें (POTENTIAL_FRICTION); मान का स्रोत: PUBLISHED, CALCULATED; चेतावनी संकेत, जैसे रखरखाव शुल्क अज्ञात (UNKNOWN_MAINTENANCE), नक्शे पर स्थान नहीं (NO_COORDINATES), मुख्य सड़क पर (ON_MAJOR_ARTERIAL)।</t>
         </is>
       </c>
     </row>
@@ -14918,7 +14918,7 @@
   </mergeCells>
   <conditionalFormatting sqref="A12:F21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"जानकारी उपलब्ध नहीं"</formula>
+      <formula>"जानकारी उपलब्ध नहीं (UNKNOWN)"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="2">
       <formula>MOD(ROW(),2)=0</formula>

</xml_diff>